<commit_message>
support filter  in index checker
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D113A64-801C-B641-8352-68D3B181828A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15740A5-6BED-40C9-84BB-8D7348EFD417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-15" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="9" r:id="rId1"/>
@@ -1873,12 +1873,6 @@
     <t>value &gt; 0 &amp;&amp; value &lt; 20</t>
   </si>
   <si>
-    <t>id=item#*.id</t>
-  </si>
-  <si>
-    <t>id=item#item.id</t>
-  </si>
-  <si>
     <t>[1]</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
@@ -1888,6 +1882,14 @@
   </si>
   <si>
     <t>@config</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>id==item#item.id</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>id==item#*.id</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
@@ -1895,11 +1897,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1928,7 +1930,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1948,7 +1950,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2234,7 +2236,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
   </cellStyles>
@@ -3160,19 +3162,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
-    <col min="5" max="5" width="45.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" customWidth="1"/>
-    <col min="8" max="9" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="16.625" customWidth="1"/>
+    <col min="4" max="4" width="25.625" customWidth="1"/>
+    <col min="5" max="5" width="45.875" customWidth="1"/>
+    <col min="6" max="6" width="18.625" customWidth="1"/>
+    <col min="8" max="9" width="12.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="42" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -3180,7 +3182,7 @@
       <c r="E1" s="43"/>
       <c r="F1" s="43"/>
     </row>
-    <row r="2" spans="1:9" ht="16">
+    <row r="2" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3209,7 +3211,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16">
+    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3238,7 +3240,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16">
+    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -3253,7 +3255,7 @@
       <c r="H4" s="34"/>
       <c r="I4" s="34"/>
     </row>
-    <row r="5" spans="1:9" ht="16">
+    <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -3282,7 +3284,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="16">
+    <row r="6" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -3299,7 +3301,7 @@
       <c r="H6" s="34"/>
       <c r="I6" s="34"/>
     </row>
-    <row r="7" spans="1:9" ht="16">
+    <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="21" t="s">
         <v>17</v>
       </c>
@@ -3328,7 +3330,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16">
+    <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
         <v>17</v>
       </c>
@@ -3351,7 +3353,7 @@
       <c r="H8" s="35"/>
       <c r="I8" s="35"/>
     </row>
-    <row r="9" spans="1:9" ht="16">
+    <row r="9" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="21" t="s">
         <v>17</v>
       </c>
@@ -3374,7 +3376,7 @@
       <c r="H9" s="35"/>
       <c r="I9" s="35"/>
     </row>
-    <row r="10" spans="1:9" ht="16">
+    <row r="10" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="21" t="s">
         <v>17</v>
       </c>
@@ -3397,7 +3399,7 @@
       <c r="H10" s="35"/>
       <c r="I10" s="35"/>
     </row>
-    <row r="11" spans="1:9" ht="16">
+    <row r="11" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="21" t="s">
         <v>17</v>
       </c>
@@ -3420,7 +3422,7 @@
       <c r="H11" s="35"/>
       <c r="I11" s="35"/>
     </row>
-    <row r="12" spans="1:9" ht="16">
+    <row r="12" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="21" t="s">
         <v>17</v>
       </c>
@@ -3443,7 +3445,7 @@
       <c r="H12" s="35"/>
       <c r="I12" s="35"/>
     </row>
-    <row r="13" spans="1:9" ht="16">
+    <row r="13" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="21" t="s">
         <v>17</v>
       </c>
@@ -3466,7 +3468,7 @@
       <c r="H13" s="35"/>
       <c r="I13" s="35"/>
     </row>
-    <row r="14" spans="1:9" ht="16">
+    <row r="14" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A14" s="21" t="s">
         <v>17</v>
       </c>
@@ -3493,7 +3495,7 @@
       </c>
       <c r="I14" s="35"/>
     </row>
-    <row r="15" spans="1:9" ht="16">
+    <row r="15" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A15" s="21" t="s">
         <v>17</v>
       </c>
@@ -3516,7 +3518,7 @@
       <c r="H15" s="35"/>
       <c r="I15" s="35"/>
     </row>
-    <row r="16" spans="1:9" ht="16">
+    <row r="16" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A16" s="21" t="s">
         <v>17</v>
       </c>
@@ -3539,7 +3541,7 @@
       <c r="H16" s="35"/>
       <c r="I16" s="35"/>
     </row>
-    <row r="17" spans="1:9" ht="16">
+    <row r="17" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A17" s="21" t="s">
         <v>17</v>
       </c>
@@ -3562,7 +3564,7 @@
       <c r="H17" s="35"/>
       <c r="I17" s="35"/>
     </row>
-    <row r="18" spans="1:9" ht="16">
+    <row r="18" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A18" s="21" t="s">
         <v>17</v>
       </c>
@@ -3585,7 +3587,7 @@
       <c r="H18" s="35"/>
       <c r="I18" s="35"/>
     </row>
-    <row r="19" spans="1:9" ht="16">
+    <row r="19" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A19" s="21" t="s">
         <v>17</v>
       </c>
@@ -3608,7 +3610,7 @@
       <c r="H19" s="35"/>
       <c r="I19" s="35"/>
     </row>
-    <row r="20" spans="1:9" ht="16">
+    <row r="20" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A20" s="21" t="s">
         <v>17</v>
       </c>
@@ -3635,7 +3637,7 @@
       </c>
       <c r="I20" s="35"/>
     </row>
-    <row r="21" spans="1:9" ht="16">
+    <row r="21" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A21" s="21" t="s">
         <v>17</v>
       </c>
@@ -3658,7 +3660,7 @@
       <c r="H21" s="35"/>
       <c r="I21" s="35"/>
     </row>
-    <row r="22" spans="1:9" ht="16">
+    <row r="22" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A22" s="21" t="s">
         <v>17</v>
       </c>
@@ -3681,7 +3683,7 @@
       <c r="H22" s="35"/>
       <c r="I22" s="35"/>
     </row>
-    <row r="23" spans="1:9" ht="16">
+    <row r="23" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A23" s="21" t="s">
         <v>17</v>
       </c>
@@ -3704,7 +3706,7 @@
       <c r="H23" s="35"/>
       <c r="I23" s="35"/>
     </row>
-    <row r="24" spans="1:9" ht="16">
+    <row r="24" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A24" s="21" t="s">
         <v>17</v>
       </c>
@@ -3740,25 +3742,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{984B885C-48D0-4D9B-AAB3-39C5F463E278}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="41"/>
     <col min="2" max="2" width="32.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="49" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="44" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
       <c r="D1" s="45"/>
       <c r="E1" s="45"/>
     </row>
-    <row r="2" spans="1:5" ht="16">
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3775,7 +3777,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3792,7 +3794,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -3801,7 +3803,7 @@
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -3818,7 +3820,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -3835,7 +3837,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="41" t="s">
         <v>17</v>
       </c>
@@ -3852,7 +3854,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="41" t="s">
         <v>17</v>
       </c>
@@ -3869,7 +3871,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="41" t="s">
         <v>17</v>
       </c>
@@ -3887,7 +3889,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="41" t="s">
         <v>17</v>
       </c>
@@ -3918,26 +3920,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.1640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" style="9" customWidth="1"/>
-    <col min="3" max="4" width="15.1640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" style="8" customWidth="1"/>
-    <col min="8" max="8" width="23.1640625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="17.125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="17.875" style="9" customWidth="1"/>
+    <col min="3" max="4" width="15.125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="26.875" style="9" customWidth="1"/>
+    <col min="6" max="6" width="8.625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.125" style="8" customWidth="1"/>
+    <col min="8" max="8" width="23.125" style="9" customWidth="1"/>
     <col min="9" max="9" width="5" style="9" customWidth="1"/>
-    <col min="10" max="10" width="46.1640625" style="9" customWidth="1"/>
+    <col min="10" max="10" width="46.125" style="9" customWidth="1"/>
     <col min="11" max="11" width="31.5" style="9" customWidth="1"/>
     <col min="12" max="12" width="8" style="9" customWidth="1"/>
-    <col min="13" max="13" width="73.6640625" style="9" customWidth="1"/>
-    <col min="14" max="14" width="13.1640625" style="9" customWidth="1"/>
-    <col min="15" max="15" width="20.6640625" style="8" customWidth="1"/>
+    <col min="13" max="13" width="73.625" style="9" customWidth="1"/>
+    <col min="14" max="14" width="13.125" style="9" customWidth="1"/>
+    <col min="15" max="15" width="20.625" style="8" customWidth="1"/>
     <col min="16" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4011,7 +4013,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="21" t="s">
         <v>22</v>
       </c>
@@ -4085,7 +4087,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
         <v>12</v>
       </c>
@@ -4141,7 +4143,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
         <v>14</v>
       </c>
@@ -4182,7 +4184,7 @@
         <v>13</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="O4" s="12" t="s">
         <v>13</v>
@@ -4215,7 +4217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
         <v>15</v>
       </c>
@@ -4287,7 +4289,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="17">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" s="24">
         <v>1001</v>
       </c>
@@ -4352,7 +4354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" s="24">
         <v>1002</v>
       </c>
@@ -4412,7 +4414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="17">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" s="24">
         <v>1003</v>
       </c>
@@ -4477,7 +4479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="17">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" s="24">
         <v>1014</v>
       </c>
@@ -4539,7 +4541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="24">
         <v>100301</v>
       </c>
@@ -4609,7 +4611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="17">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="24">
         <v>100302</v>
       </c>
@@ -4669,7 +4671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:24" s="20" customFormat="1" ht="17">
+    <row r="12" spans="1:24" s="20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="26">
         <v>100303</v>
       </c>
@@ -4729,7 +4731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="17">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="24">
         <v>100001</v>
       </c>
@@ -4789,7 +4791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" s="24">
         <v>100002</v>
       </c>
@@ -4849,7 +4851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" s="24">
         <v>100003</v>
       </c>
@@ -4911,7 +4913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="17">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" s="24">
         <v>100304</v>
       </c>
@@ -4971,7 +4973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="17">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="24">
         <v>1013</v>
       </c>
@@ -5043,26 +5045,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:W16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.1640625" style="9" customWidth="1"/>
-    <col min="2" max="3" width="17.83203125" style="9" customWidth="1"/>
-    <col min="4" max="5" width="15.1640625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="17.125" style="9" customWidth="1"/>
+    <col min="2" max="3" width="17.875" style="9" customWidth="1"/>
+    <col min="4" max="5" width="15.125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="19.875" style="9" customWidth="1"/>
     <col min="7" max="7" width="28" style="9" customWidth="1"/>
-    <col min="8" max="8" width="15.1640625" style="9" customWidth="1"/>
-    <col min="9" max="9" width="23.1640625" style="9" customWidth="1"/>
-    <col min="10" max="10" width="16.1640625" style="9" customWidth="1"/>
-    <col min="11" max="11" width="63.1640625" style="9" customWidth="1"/>
-    <col min="12" max="12" width="20.1640625" style="9" customWidth="1"/>
-    <col min="13" max="13" width="13.1640625" style="9" customWidth="1"/>
+    <col min="8" max="8" width="15.125" style="9" customWidth="1"/>
+    <col min="9" max="9" width="23.125" style="9" customWidth="1"/>
+    <col min="10" max="10" width="16.125" style="9" customWidth="1"/>
+    <col min="11" max="11" width="63.125" style="9" customWidth="1"/>
+    <col min="12" max="12" width="20.125" style="9" customWidth="1"/>
+    <col min="13" max="13" width="13.125" style="9" customWidth="1"/>
     <col min="14" max="14" width="9" style="9"/>
-    <col min="15" max="15" width="13.1640625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="13.125" style="9" customWidth="1"/>
     <col min="16" max="16" width="11" style="9" customWidth="1"/>
     <col min="17" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5130,7 +5132,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -5198,7 +5200,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -5249,7 +5251,7 @@
       </c>
       <c r="W3" s="1"/>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -5318,7 +5320,7 @@
       </c>
       <c r="W4" s="12"/>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -5384,7 +5386,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="1:23">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <f t="shared" ref="A6:A16" si="0">200000+C6*100+D6</f>
         <v>200101</v>
@@ -5441,7 +5443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <f t="shared" si="0"/>
         <v>200102</v>
@@ -5497,7 +5499,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <f t="shared" si="0"/>
         <v>200103</v>
@@ -5556,7 +5558,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <f t="shared" si="0"/>
         <v>200104</v>
@@ -5612,7 +5614,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <f t="shared" si="0"/>
         <v>200105</v>
@@ -5668,7 +5670,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <f t="shared" si="0"/>
         <v>200106</v>
@@ -5724,7 +5726,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:23">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
         <f t="shared" si="0"/>
         <v>200107</v>
@@ -5780,7 +5782,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
         <f t="shared" si="0"/>
         <v>200201</v>
@@ -5839,7 +5841,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:23">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="9">
         <f t="shared" si="0"/>
         <v>200202</v>
@@ -5898,7 +5900,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <f t="shared" si="0"/>
         <v>200203</v>
@@ -5957,7 +5959,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:23">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="9">
         <f t="shared" si="0"/>
         <v>200204</v>
@@ -6027,16 +6029,16 @@
     <tabColor theme="5" tint="0.39915158543656726"/>
   </sheetPr>
   <dimension ref="A1:I19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="17.1640625" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" style="9" customWidth="1"/>
-    <col min="4" max="7" width="17.1640625" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" customWidth="1"/>
-    <col min="9" max="9" width="13.1640625" style="9" customWidth="1"/>
+    <col min="1" max="2" width="17.125" customWidth="1"/>
+    <col min="3" max="3" width="15.125" style="9" customWidth="1"/>
+    <col min="4" max="7" width="17.125" customWidth="1"/>
+    <col min="8" max="8" width="20.125" customWidth="1"/>
+    <col min="9" max="9" width="13.125" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6065,7 +6067,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="16.5">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6094,7 +6096,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6115,7 +6117,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6144,7 +6146,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="16.5">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -6173,7 +6175,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>177</v>
       </c>
@@ -6202,7 +6204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>183</v>
       </c>
@@ -6231,7 +6233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>188</v>
       </c>
@@ -6260,7 +6262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>193</v>
       </c>
@@ -6289,7 +6291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
@@ -6300,7 +6302,7 @@
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
@@ -6311,7 +6313,7 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -6322,7 +6324,7 @@
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -6333,7 +6335,7 @@
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
@@ -6344,7 +6346,7 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="4"/>
       <c r="B15" s="5"/>
       <c r="C15" s="6"/>
@@ -6355,7 +6357,7 @@
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="4"/>
       <c r="B16" s="5"/>
       <c r="C16" s="6"/>
@@ -6366,7 +6368,7 @@
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="4"/>
       <c r="B17" s="5"/>
       <c r="C17" s="6"/>
@@ -6377,7 +6379,7 @@
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
       <c r="B18" s="5"/>
       <c r="C18" s="6"/>
@@ -6388,7 +6390,7 @@
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="4"/>
       <c r="B19" s="5"/>
       <c r="C19" s="6"/>
@@ -6412,17 +6414,17 @@
     <tabColor theme="5" tint="0.39915158543656726"/>
   </sheetPr>
   <dimension ref="A1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="17.1640625" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="17.125" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="17.1640625" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" style="9" customWidth="1"/>
-    <col min="4" max="7" width="17.1640625" customWidth="1"/>
-    <col min="8" max="9" width="25.6640625" customWidth="1"/>
-    <col min="10" max="10" width="13.1640625" style="9" customWidth="1"/>
-    <col min="11" max="16377" width="17.1640625" customWidth="1"/>
+    <col min="1" max="2" width="17.125" customWidth="1"/>
+    <col min="3" max="3" width="15.125" style="9" customWidth="1"/>
+    <col min="4" max="7" width="17.125" customWidth="1"/>
+    <col min="8" max="9" width="25.625" customWidth="1"/>
+    <col min="10" max="10" width="13.125" style="9" customWidth="1"/>
+    <col min="11" max="16377" width="17.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6454,7 +6456,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.5">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6486,7 +6488,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16.5">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6508,7 +6510,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16.5">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6531,16 +6533,16 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16.5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -6572,7 +6574,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>200</v>
       </c>
@@ -6604,7 +6606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>202</v>
       </c>
@@ -6636,7 +6638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>206</v>
       </c>
@@ -6668,7 +6670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>210</v>
       </c>
@@ -6700,7 +6702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
@@ -6712,7 +6714,7 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
@@ -6724,7 +6726,7 @@
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -6736,7 +6738,7 @@
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -6748,7 +6750,7 @@
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
@@ -6760,19 +6762,19 @@
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="J15" s="6"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="J16" s="6"/>
     </row>
-    <row r="17" spans="10:10">
+    <row r="17" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J17" s="6"/>
     </row>
-    <row r="18" spans="10:10">
+    <row r="18" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J18" s="6"/>
     </row>
-    <row r="19" spans="10:10">
+    <row r="19" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J19" s="6"/>
     </row>
   </sheetData>
@@ -6785,18 +6787,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="10.625" customWidth="1"/>
     <col min="5" max="5" width="29" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="9" max="9" width="35.6640625" customWidth="1"/>
-    <col min="10" max="10" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.875" customWidth="1"/>
+    <col min="7" max="7" width="16.625" customWidth="1"/>
+    <col min="9" max="9" width="35.625" customWidth="1"/>
+    <col min="10" max="10" width="21.875" customWidth="1"/>
     <col min="12" max="12" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16">
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6834,7 +6836,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16">
+    <row r="2" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6872,7 +6874,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16">
+    <row r="3" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6896,7 +6898,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16">
+    <row r="4" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6934,7 +6936,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16">
+    <row r="5" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -6972,7 +6974,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16">
+    <row r="6" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>215</v>
       </c>
@@ -7006,7 +7008,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="16">
+    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>221</v>
       </c>
@@ -7040,7 +7042,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16">
+    <row r="8" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>226</v>
       </c>
@@ -7074,7 +7076,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="16">
+    <row r="9" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>231</v>
       </c>

</xml_diff>

<commit_message>
use $ to get current cell value
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB5CD89-8AB6-3148-987F-0B4A6C468DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AAAA6AB-38A7-CF4E-AF61-BE2B7A38F754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="9" r:id="rId1"/>
@@ -1870,9 +1870,6 @@
     <t>{200106}</t>
   </si>
   <si>
-    <t>value &gt; 0 &amp;&amp; value &lt; 20</t>
-  </si>
-  <si>
     <t>[1]</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
@@ -1897,6 +1894,9 @@
   </si>
   <si>
     <t>key2=MAIN==#main.type&amp;condition=mainline_event</t>
+  </si>
+  <si>
+    <t>$ &gt; 0 &amp;&amp; $ &lt; 20</t>
   </si>
 </sst>
 </file>
@@ -3180,7 +3180,7 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="42" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -3278,7 +3278,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G5" s="33" t="s">
         <v>13</v>
@@ -3759,7 +3759,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="44" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
@@ -4157,10 +4157,10 @@
         <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
@@ -4190,7 +4190,7 @@
         <v>13</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="O4" s="12" t="s">
         <v>13</v>
@@ -6044,7 +6044,7 @@
     <col min="9" max="9" width="13.1640625" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6073,7 +6073,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="16.5">
+    <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6102,7 +6102,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5">
+    <row r="3" spans="1:9">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6123,7 +6123,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5">
+    <row r="4" spans="1:9">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6152,7 +6152,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="16.5">
+    <row r="5" spans="1:9">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -6430,7 +6430,7 @@
     <col min="11" max="16377" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6462,7 +6462,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.5">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6494,7 +6494,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16.5">
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16.5">
+    <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6539,16 +6539,16 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>259</v>
-      </c>
       <c r="J4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16.5">
+    <row r="5" spans="1:10">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>

</xml_diff>